<commit_message>
docs: Team1 V2 — 12→14 周，拆分 W3~W5 过载段并独立 DevOps Sprint
- 原 S2（W3~W5 功能+就绪混排）拆为：S2 功能开发（W3~W4，纯功能）+
  S3 DevOps与就绪（W5~W6：CD 多环境/四道门禁/发布包/回退演练/监控/预跑），
  R1 上线移至 W7
- R2 同理：S5 扩为 W10~W13（全量+合规+连接器+就绪，多一周），R2 上线 W14
- 总工期 12→14 周（+2 周）；人天口径不变（150），节奏舒展不加范围
- 5 个 Sprint + 周计划 42 块重排

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/report/Team1.xlsx
+++ b/report/Team1.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;￥&quot;#,##0;&quot;￥&quot;\-#,##0"/>
   </numFmts>
-  <fonts count="58">
+  <fonts count="59">
     <font>
       <name val="Microsoft YaHei"/>
       <charset val="134"/>
@@ -396,8 +396,14 @@
       <color rgb="007c3aed"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Microsoft YaHei"/>
+      <b val="1"/>
+      <color rgb="00ca8a04"/>
+      <sz val="9.199999999999999"/>
+    </font>
   </fonts>
-  <fills count="47">
+  <fills count="48">
     <fill>
       <patternFill/>
     </fill>
@@ -666,6 +672,11 @@
         <fgColor rgb="00FFEDD5"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="17">
     <border>
@@ -1022,7 +1033,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1163,6 +1174,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="57" fillId="43" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="58" fillId="47" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2093,7 +2107,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" style="18" min="1" max="1"/>
@@ -2109,14 +2123,14 @@
     <row r="1">
       <c r="A1" s="20" t="inlineStr">
         <is>
-          <t>B2 湖仓归档平台 · 3 人团队执行计划（BA + Dev + QA · 双 Release 对半 · AI Vibe Coding）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" s="18">
+          <t>B2 湖仓归档平台 · 3 人团队执行计划 V2（14 周 · 双 Release · AI Vibe Coding）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="32" customHeight="1" s="18">
       <c r="A2" s="21" t="inlineStr">
         <is>
-          <t>R1 归档检索平台（W1~W6）：存量迁移 + 检索/权限/审计 → W6 Go-Live #1 · R2 治理合规完整版（W7~W12）：治理/生命周期/安全/合规报表 + 全量迁移 + 文档 → W12 Go-Live #2 + 项目结束 · CC（Caring Center）单系统贯穿验证</t>
+          <t>V2 调整：原 W3~W5 工作过载，拆为「功能开发（W3~W4）+ DevOps与就绪（W5~W6）」两个 Sprint，R1 上线移至 W7；R2 同理多拆一周，上线 W14。R1 = W1~W7 / R2 = W8~W14（各 +1 周，共 14 周）· CC 单系统贯穿</t>
         </is>
       </c>
     </row>
@@ -2187,22 +2201,22 @@
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
-          <t>【BA】① BRD 定稿（数据流图+保留期矩阵+PII 分级+检索权限矩阵）② CC 垃圾表剔除标准与首批 50 表清单确认 【DEV-Wade】③ 架构定稿 + 资源申请（区域=境内）+ 资源验收 + UC 初始化（arch_cc）④ 前后端骨架 + Azure DevOps Pipelines CI ⑤ SeaTunnel PoC（CC 抽样 10 表端到端）+ 1253 表扫描分类 ⑥【01】首批 50 表批量导入（分片/限速/断点）+ 配置生成器 v1 【QA】⑦ 测试计划（8 域）+ 架构图×2（上下文/容器）+ 文档模板 ⑧ 迁移对账测试设计</t>
+          <t>【BA】① BRD 定稿（数据流图+保留期矩阵+PII 分级+检索权限矩阵）② CC 垃圾表标准与首批 50 表清单 【DEV】③ 架构定稿+资源申请+验收+UC 初始化 ④ 前后端骨架+CI 骨架 ⑤ SeaTunnel PoC（10 表端到端）+ 1253 表分类 ⑥【01】50 表批量导入+生成器 v1 【QA】⑦ 测试计划（8 域）+ 架构图×2 + 文档模板</t>
         </is>
       </c>
       <c r="F5" s="28" t="inlineStr">
         <is>
-          <t>★ W2：CC PoC 端到端 + BRD 签字 + 50 表入 RAW + 登录页可访问</t>
+          <t>★ W2：PoC 端到端 + BRD 签字 + 50 表入 RAW</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
         <is>
-          <t>CC 账号/白名单周期；Wade 一人扛三角色串行风险；1253 表审表量</t>
+          <t>CC 账号周期；Wade 串行压力</t>
         </is>
       </c>
       <c r="H5" s="30" t="inlineStr">
         <is>
-          <t>① CC 只读账号（W1）② 垃圾表标准 ③ 50 表清单（W2 末）</t>
+          <t>① CC 账号 ② 垃圾表标准 ③ 50 表清单</t>
         </is>
       </c>
     </row>
@@ -2216,37 +2230,37 @@
       <c r="B6" s="31" t="inlineStr">
         <is>
           <t>Sprint 2
-检索增强+就绪</t>
+检索与权限</t>
         </is>
       </c>
       <c r="C6" s="25" t="inlineStr">
         <is>
-          <t>W3~W5</t>
+          <t>W3~W4</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>检索/权限/审计端到端 + R1 上线就绪</t>
+          <t>检索/权限/审计 功能开发（纯功能，不做上线准备）</t>
         </is>
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>【DEV-Wade】【05】① 配置化检索页 + 预览（SAS）+ 导出【08】② RBAC 五角色 + UC GRANT + 掩码函数（权限三态）③ SSO JWT Claims ④【06】审计埋点【07】⑤ 连接器模板 v1 ⑥ SERVE 热表物化【安全】⑦ 四道 CI 门禁 【BA】⑧ PII 字段标记 + 预览范围确认 ⑨ R1 验收 + UAT #1 脚本【QA】⑩ 功能/安全测试执行 ⑪ R1 文档 50%（用户手册检索章节）【就绪 W5】⑫ 发布包+回退演练+UAT 预演+迁移预跑+就绪检查</t>
+          <t>【DEV】【05】① 配置化检索页 ② 预览（SAS）③ 导出【08】④ RBAC 五角色 CRUD+鉴权 ⑤ UC GRANT+掩码函数（权限三态）⑥ SERVE 物化 【06】⑦ 审计埋点【07】⑧ 连接器模板 v1【安全】⑨ 依赖扫描+SAST 门禁 【BA】⑩ PII 字段标记+预览范围 ⑪ R1 功能验收 【QA】⑫ 功能/安全测试 ⑬ 文档 50%</t>
         </is>
       </c>
       <c r="F6" s="28" t="inlineStr">
         <is>
-          <t>★ W5 末：R1 上线就绪检查 100%（发布包/预演/回退/预跑全绿）</t>
+          <t>★ W4：R1 功能全部 Done（登录→检索→预览→导出+权限三态）</t>
         </is>
       </c>
       <c r="G6" s="29" t="inlineStr">
         <is>
-          <t>Wade 任务密度最高的一段；权限三态联调复杂</t>
+          <t>功能密度仍高但不再混上线准备；掩码/三态是硬骨头</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
         <is>
-          <t>① PII 标记（W3）② 性能标准 P95&lt;5s ③ UAT 预演排期</t>
+          <t>① PII 标记（W3）② 性能标准</t>
         </is>
       </c>
     </row>
@@ -2257,219 +2271,263 @@
 归档检索平台</t>
         </is>
       </c>
-      <c r="B7" s="31" t="inlineStr">
-        <is>
-          <t>Sprint 2
-检索增强+就绪</t>
+      <c r="B7" s="50" t="inlineStr">
+        <is>
+          <t>Sprint 3
+DevOps+R1就绪</t>
         </is>
       </c>
       <c r="C7" s="25" t="inlineStr">
         <is>
-          <t>W6</t>
+          <t>W5~W6</t>
         </is>
       </c>
       <c r="D7" s="26" t="inlineStr">
         <is>
-          <t>R1 上线周：发布 → UAT → Go-Live #1</t>
+          <t>DevOps + R1 上线就绪（独立 Sprint，不再挤占功能期）</t>
         </is>
       </c>
       <c r="E7" s="27" t="inlineStr">
         <is>
-          <t>【DEV】① 生产发布（就绪包一键发布+Environments 审批）② CC 50 表生产迁移+对账 ③ P1 当日清 【BA】④ UAT #1 正式主持（检索/预览/导出/权限/SSO/审计 → 签字）⑤ Go/No-Go 需求侧 【QA】⑥ 上线记录 + R1 审批材料提交 ⑦ 48h 值守三角色轮值</t>
+          <t>【DEV·DevOps】① CD 流水线完善（Helm 多环境 Dev/Staging/Prod + Environments 审批流）② 四道安全门禁全量上线（gitleaks/Trivy）③ 生产发布包（一键发布就绪）④ 回退预案与演练 ⑤ 监控告警就绪（App Insights+Dashboard）⑥ CC 迁移预跑+Runbook 【BA】⑦ UAT #1 脚本+预演主持 【QA】⑧ R1 文档冲刺（用户手册/运维手册 70%）⑨ 上线 Checklist ⑩ W6 末就绪检查</t>
         </is>
       </c>
       <c r="F7" s="28" t="inlineStr">
         <is>
-          <t>★ W6：Go-Live #1 —— CC 可查、有权限、有审计（Release 1 交付）</t>
+          <t>★ W6 末：R1 就绪检查 100%（DevOps 就绪/预演/回退/预跑全绿）</t>
         </is>
       </c>
       <c r="G7" s="29" t="inlineStr">
         <is>
-          <t>三人全上线值守（轮值缓解）；审批受理时长</t>
+          <t>DevOps 环境问题（AKS 权限/ACR 网络）；预演排期</t>
         </is>
       </c>
       <c r="H7" s="30" t="inlineStr">
         <is>
-          <t>① Go-Live #1 窗口 ② UAT #1 签字人</t>
+          <t>① 生产环境权限 ② 预演排期 ③ 迁移窗口</t>
         </is>
       </c>
     </row>
     <row r="8" ht="132" customHeight="1" s="18">
-      <c r="A8" s="32" t="inlineStr">
+      <c r="A8" s="23" t="inlineStr">
+        <is>
+          <t>Release 1
+归档检索平台</t>
+        </is>
+      </c>
+      <c r="B8" s="50" t="inlineStr">
+        <is>
+          <t>Sprint 3
+DevOps+R1就绪</t>
+        </is>
+      </c>
+      <c r="C8" s="25" t="inlineStr">
+        <is>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>R1 上线周：发布 → UAT → Go-Live #1（仅执行）</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>【DEV】① 生产发布（就绪包+审批）② CC 50 表生产迁移+对账 ③ P1 当日清 【BA】④ UAT #1 正式主持（签字）⑤ Go/No-Go 【QA】⑥ 上线记录+R1 审批材料提交 ⑦ 48h 值守三角色轮值</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="inlineStr">
+        <is>
+          <t>★ W7：Go-Live #1 —— CC 可查、有权限、有审计（Release 1 交付）</t>
+        </is>
+      </c>
+      <c r="G8" s="29" t="inlineStr">
+        <is>
+          <t>依赖 W6 就绪检查通过</t>
+        </is>
+      </c>
+      <c r="H8" s="30" t="inlineStr">
+        <is>
+          <t>① Go 窗口 ② UAT 签字人</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="132" customHeight="1" s="18">
+      <c r="A9" s="32" t="inlineStr">
         <is>
           <t>Release 2
 治理合规完整版</t>
         </is>
       </c>
-      <c r="B8" s="33" t="inlineStr">
-        <is>
-          <t>Sprint 3
+      <c r="B9" s="33" t="inlineStr">
+        <is>
+          <t>Sprint 4
 治理+安全</t>
         </is>
       </c>
-      <c r="C8" s="25" t="inlineStr">
-        <is>
-          <t>W7~W9</t>
-        </is>
-      </c>
-      <c r="D8" s="26" t="inlineStr">
-        <is>
-          <t>治理 + 生命周期 + 安全管控（R2 功能主体）</t>
-        </is>
-      </c>
-      <c r="E8" s="27" t="inlineStr">
-        <is>
-          <t>【DEV-Wade】【02】① 增量接入（watermark）+ 冷数据自动转冷 ② 元数据标准界面 【03】③ 处置引擎（DROP PARTITION+VACUUM）+ Legal Hold + 归档模型 ④ 处置/Hold 界面 【04】⑤ 加密（CMK+字段级+轮转）+ 脱敏 + 境内驻留核查 ⑥ ADLS 分层+生命周期+Compaction 【07】⑦ 连接器模板库（MySQL+文件源）+ 连接管理界面【08】⑧ 行级隔离验证 【BA】⑨ Legal Hold 触发条件定稿（法务）⑩ 增量频率/冷数据标准 【QA】⑪ 处置全链路 E2E（1 天保留期→到期→Hold→处置→审计）⑫ 掩码旁路/越权测试 ⑬ 文档 60%</t>
-        </is>
-      </c>
-      <c r="F8" s="28" t="inlineStr">
-        <is>
-          <t>★ W8：处置全链路通过+脱敏三态+驻留核查；★ W9：越权全拦截+新源 30 分钟接入</t>
-        </is>
-      </c>
-      <c r="G8" s="29" t="inlineStr">
-        <is>
-          <t>处置不可逆需沙箱验证；加密/驻留须人工复核（Wade 自查=风险）</t>
-        </is>
-      </c>
-      <c r="H8" s="30" t="inlineStr">
-        <is>
-          <t>① Legal Hold 审批人 ② 保留期底线 ③ 实时指标验收</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="132" customHeight="1" s="18">
-      <c r="A9" s="32" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
+        <is>
+          <t>W8~W9</t>
+        </is>
+      </c>
+      <c r="D9" s="26" t="inlineStr">
+        <is>
+          <t>治理 + 生命周期 + 安全管控（R2 功能主体一）</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>【DEV】【02】① 增量接入+冷数据转冷 ② 元数据标准界面【03】③ 处置引擎+Legal Hold+归档模型 ④ 处置/Hold 界面 【04】⑤ 加密+脱敏+驻留核查 ⑥ ADLS 分层+Compaction【07】⑦ 连接器模板库 【BA】⑧ Hold 条件定稿（法务）【QA】⑨ 处置 E2E+安全测试 ⑩ 文档 60%</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="inlineStr">
+        <is>
+          <t>★ W9：处置全链路+脱敏三态+驻留核查通过</t>
+        </is>
+      </c>
+      <c r="G9" s="29" t="inlineStr">
+        <is>
+          <t>处置不可逆；加密需人工复核</t>
+        </is>
+      </c>
+      <c r="H9" s="30" t="inlineStr">
+        <is>
+          <t>① Hold 审批人 ② 保留期底线 ③ 实时指标</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="132" customHeight="1" s="18">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>Release 2
 治理合规完整版</t>
         </is>
       </c>
-      <c r="B9" s="34" t="inlineStr">
-        <is>
-          <t>Sprint 4
-全量+合规+就绪</t>
-        </is>
-      </c>
-      <c r="C9" s="25" t="inlineStr">
-        <is>
-          <t>W10~W11</t>
-        </is>
-      </c>
-      <c r="D9" s="26" t="inlineStr">
-        <is>
-          <t>CC 全量迁移 + 合规报表 + R2 上线就绪</t>
-        </is>
-      </c>
-      <c r="E9" s="27" t="inlineStr">
-        <is>
-          <t>【DEV-Wade】【01】① CC 全量 1253 表分批迁移（600~800 有效表）+ 逐批对账 【06】② 合规报表（等保/个保法对照+导出）③ 全量回归（R1+R2）④ R2 发布包+回退演练 ⑤ 安全终检（四门禁+渗透配合）⑥ 迁移预跑+窗口预约 【BA】⑦ 全量范围最终确认（签字）⑧ 合规报表口径对齐（法务）⑨ UAT #2 脚本 【QA】⑩ 文档冲刺（7 套 80%→终稿）+ 审批材料 ⑪ 连接器兼容矩阵 + 口径验证 ⑫ W11 末就绪检查</t>
-        </is>
-      </c>
-      <c r="F9" s="28" t="inlineStr">
-        <is>
-          <t>★ W10：CC 全量对账 100%；★ W11 末：R2 就绪检查 100%</t>
-        </is>
-      </c>
-      <c r="G9" s="29" t="inlineStr">
-        <is>
-          <t>全量迁移时长不可控；文档冲刺与就绪并行（QA 压力最大）</t>
-        </is>
-      </c>
-      <c r="H9" s="30" t="inlineStr">
-        <is>
-          <t>① CC 数据量实测 ② 迁移窗口 ③ 报表口径签字人</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="132" customHeight="1" s="18">
-      <c r="A10" s="32" t="inlineStr">
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5
+全量+合规+R2就绪</t>
+        </is>
+      </c>
+      <c r="C10" s="25" t="inlineStr">
+        <is>
+          <t>W10~W13</t>
+        </is>
+      </c>
+      <c r="D10" s="26" t="inlineStr">
+        <is>
+          <t>CC 全量 + 合规报表 + 连接器完善 + R2 就绪（多一周，不再挤）</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>【DEV】【01】① CC 全量 1253 表分批迁移+逐批对账【06】② 合规报表【07】③ 连接器运行监控+连接管理界面【08】④ 行级隔离验证 【就绪 W12~13】⑤ 全量回归（R1+R2）⑥ R2 发布包+回退演练 ⑦ 安全终检（四门禁+渗透）⑧ 迁移预跑+窗口预约 【BA】⑨ 全量范围签字 ⑩ 报表口径对齐 ⑪ UAT #2 脚本+预演 【QA】⑫ 文档冲刺（7 套终稿）+审批材料 ⑬ 兼容矩阵 ⑭ W13 末就绪检查</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="inlineStr">
+        <is>
+          <t>★ W11：全量对账 100%；★ W13 末：R2 就绪检查 100%</t>
+        </is>
+      </c>
+      <c r="G10" s="29" t="inlineStr">
+        <is>
+          <t>全量迁移时长；文档冲刺与就绪并行</t>
+        </is>
+      </c>
+      <c r="H10" s="30" t="inlineStr">
+        <is>
+          <t>① 数据量实测 ② 迁移窗口 ③ 报表口径签字</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="132" customHeight="1" s="18">
+      <c r="A11" s="32" t="inlineStr">
         <is>
           <t>Release 2
 治理合规完整版</t>
         </is>
       </c>
-      <c r="B10" s="34" t="inlineStr">
-        <is>
-          <t>Sprint 4
-全量+合规+就绪</t>
-        </is>
-      </c>
-      <c r="C10" s="25" t="inlineStr">
-        <is>
-          <t>W12</t>
-        </is>
-      </c>
-      <c r="D10" s="26" t="inlineStr">
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t>Sprint 5
+全量+合规+R2就绪</t>
+        </is>
+      </c>
+      <c r="C11" s="25" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
         <is>
           <t>R2 上线周 + 收尾：Go-Live #2 → 项目结束</t>
         </is>
       </c>
-      <c r="E10" s="27" t="inlineStr">
-        <is>
-          <t>【DEV】① R2 生产发布（治理/安全/合规，增量发布不中断 R1）② CC 生产全量迁移收尾+终版对账 ③ P1 当日清 【BA】④ UAT #2 正式主持（处置/Hold/脱敏/报表 → 签字）⑤ Go/No-Go 【QA】⑥ 审批材料提交（完整版）⑦ 文档终版归档（7 套）⑧ 上线验证与稳定性报告 → 项目结束</t>
-        </is>
-      </c>
-      <c r="F10" s="28" t="inlineStr">
-        <is>
-          <t>★ W12：Go-Live #2（完整版）+ 交付物归档 → 项目结束</t>
-        </is>
-      </c>
-      <c r="G10" s="29" t="inlineStr">
-        <is>
-          <t>上线+文档+收尾三线并行在 W12；全量迁移收尾跨窗口</t>
-        </is>
-      </c>
-      <c r="H10" s="30" t="inlineStr">
-        <is>
-          <t>① Go-Live #2 窗口 ② UAT #2 签字人 ③ 文档确认</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="26" customHeight="1" s="18">
-      <c r="A12" s="35" t="inlineStr">
-        <is>
-          <t>团队：3 人 —— BA（Mandy，50% 投入）/ DEV（Wade，全职，承担架构+数据工程+全栈 DevOps 三角色）/ QA（全职，测试+SLC 文档）</t>
+      <c r="E11" s="27" t="inlineStr">
+        <is>
+          <t>【DEV】① R2 生产发布（增量不中断 R1）② CC 生产全量迁移收尾+终版对账 ③ P1 当日清 【BA】④ UAT #2 正式主持（签字）⑤ Go/No-Go 【QA】⑥ 审批材料提交 ⑦ 文档终版归档（7 套）⑧ 稳定性报告 → 项目结束</t>
+        </is>
+      </c>
+      <c r="F11" s="28" t="inlineStr">
+        <is>
+          <t>★ W14：Go-Live #2（完整版）+ 交付物归档 → 项目结束</t>
+        </is>
+      </c>
+      <c r="G11" s="29" t="inlineStr">
+        <is>
+          <t>上线+文档+收尾并行；迁移收尾跨窗口</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>① Go 窗口 ② UAT 签字人 ③ 文档确认</t>
         </is>
       </c>
     </row>
     <row r="13" ht="26" customHeight="1" s="18">
       <c r="A13" s="35" t="inlineStr">
         <is>
-          <t>结构：双 Release 对半（R1 W1~W6 / R2 W7~W12），各自"功能→就绪→上线"闭环，上线各占最后一周（W6/W12）</t>
+          <t>V2 变更：原「W3~W5 检索增强+就绪」一个 Sprint 拆为两个 —— S2 功能开发（W3~W4，纯功能）+ S3 DevOps与就绪（W5~W6），R1 上线 W7</t>
         </is>
       </c>
     </row>
     <row r="14" ht="26" customHeight="1" s="18">
       <c r="A14" s="35" t="inlineStr">
         <is>
-          <t>人天：BA 20 + DEV 100 + QA 30 = 150 人天（12 周）；人力费用 = 132,000 + 390,000 + 75,000 = ¥597,000（按 Team1 表单价）</t>
+          <t>R2 同理：原「W10~W11 全量+就绪」扩为 W10~W13（多一周），R2 上线 W14。总工期 12 → 14 周（+2 周）</t>
         </is>
       </c>
     </row>
     <row r="15" ht="26" customHeight="1" s="18">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>与 5 人版差异：DEV 集中 Wade 一人（风险↑），用 AI Vibe Coding 提效；BA 兼测试协调；无独立架构评审——建议 W1/W5 两个节点请平台团队做外部 sanity check</t>
+          <t>人天口径：仍按 Team1 表（BA 20 + DEV 100 + QA 30 = 150 人天）；+2 周主要为 DevOps/就绪/缓冲的节奏舒展，不增功能范围</t>
         </is>
       </c>
     </row>
     <row r="16" ht="26" customHeight="1" s="18">
       <c r="A16" s="35" t="inlineStr">
         <is>
-          <t>W7~W11 期间 R1 已在生产运行，R2 上线为增量发布不中断服务</t>
+          <t>团队与风险不变：Mandy·BA（50%）/ Wade·DEV（全开发，🤖 AI 提效）/ QA；无独立架构评审——W1/W5/W12 三个节点请平台团队外部 sanity check</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="26" customHeight="1" s="18">
+      <c r="A17" s="35" t="inlineStr">
+        <is>
+          <t>上线只占 W7 / W14 最后一周；W8~W13 期间 R1 已在生产运行，R2 增量发布不中断服务</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="7">
-    <mergeCell ref="A12:H12"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
     <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A17:H17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2481,14 +2539,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G96"/>
+  <dimension ref="A1:G105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="18" min="1" max="1"/>
     <col width="8" customWidth="1" style="18" min="2" max="2"/>
     <col width="6" customWidth="1" style="18" min="3" max="3"/>
     <col width="13" customWidth="1" style="18" min="4" max="4"/>
-    <col width="66" customWidth="1" style="18" min="5" max="5"/>
+    <col width="64" customWidth="1" style="18" min="5" max="5"/>
     <col width="26" customWidth="1" style="18" min="6" max="6"/>
     <col width="20" customWidth="1" style="18" min="7" max="7"/>
   </cols>
@@ -2496,14 +2554,14 @@
     <row r="1">
       <c r="A1" s="36" t="inlineStr">
         <is>
-          <t>周计划明细 · 3 人 × 12 周（BA·Mandy / DEV·Wade / QA · 双 Release · 上线仅 W6/W12）</t>
+          <t>周计划明细 · 3 人 × 14 周（W3~W4 纯功能 / W5~W6 DevOps就绪 / W7 上线 · R2 同理 / W14 上线收尾）</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="37" t="inlineStr">
         <is>
-          <t>🤖 = AI Vibe Coding 提效标注（主要落在 DEV-Wade 任务）· 外部依赖为不可压缩物理时间</t>
+          <t>🤖 = AI 提效标注 · BA·Mandy / DEV·Wade / QA · 外部依赖为不可压缩时间</t>
         </is>
       </c>
     </row>
@@ -2567,12 +2625,12 @@
       </c>
       <c r="E5" s="41" t="inlineStr">
         <is>
-          <t>• 【8 域需求访谈】业务方×2 场 + 合规法务×1 场（保留期/PII/Legal Hold）</t>
+          <t>• 【8 域需求访谈】业务方×2 + 合规法务×1（保留期/PII/Legal Hold）</t>
         </is>
       </c>
       <c r="F5" s="42" t="inlineStr">
         <is>
-          <t>BRD 初稿；CC 剔除规则</t>
+          <t>BRD 初稿；剔除规则</t>
         </is>
       </c>
       <c r="G5" s="29" t="inlineStr">
@@ -2588,7 +2646,7 @@
       <c r="D6" s="44" t="n"/>
       <c r="E6" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 BRD 起稿：数据流图 + 归档范围矩阵 + PII 分级 + 检索权限矩阵</t>
+          <t>• 🤖 BRD 起稿：数据流图+归档范围矩阵+PII 分级+检索权限矩阵</t>
         </is>
       </c>
       <c r="F6" s="43" t="n"/>
@@ -2601,7 +2659,7 @@
       <c r="D7" s="44" t="n"/>
       <c r="E7" s="41" t="inlineStr">
         <is>
-          <t>• CC 接入范围初定：1253 表垃圾表剔除标准与业务方对齐</t>
+          <t>• CC 垃圾表剔除标准与业务方对齐</t>
         </is>
       </c>
       <c r="F7" s="43" t="n"/>
@@ -2630,12 +2688,12 @@
       </c>
       <c r="E8" s="41" t="inlineStr">
         <is>
-          <t>• 架构文档定稿（湖仓分层+UC 授权+存储分层）+ 资源申请单（区域=境内）</t>
+          <t>• 架构文档定稿 + 资源申请单（区域=境内）+ CC 账号/白名单申请（D1）</t>
         </is>
       </c>
       <c r="F8" s="42" t="inlineStr">
         <is>
-          <t>架构 V1；申请单；骨架+CI</t>
+          <t>架构 V1；骨架+CI</t>
         </is>
       </c>
       <c r="G8" s="29" t="inlineStr">
@@ -2651,20 +2709,20 @@
       <c r="D9" s="46" t="n"/>
       <c r="E9" s="41" t="inlineStr">
         <is>
-          <t>• CC 只读账号 + NAT 白名单申请（D1 启动）</t>
+          <t>• 🤖 CC 1253 表扫描分类脚本</t>
         </is>
       </c>
       <c r="F9" s="43" t="n"/>
       <c r="G9" s="43" t="n"/>
     </row>
-    <row r="10" ht="30" customHeight="1" s="18">
+    <row r="10" ht="22" customHeight="1" s="18">
       <c r="A10" s="43" t="n"/>
       <c r="B10" s="43" t="n"/>
       <c r="C10" s="43" t="n"/>
       <c r="D10" s="46" t="n"/>
       <c r="E10" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 CC 1253 表扫描分类脚本 + 前后端骨架 + Azure DevOps Pipelines CI</t>
+          <t>• 🤖 前后端骨架 + CI 骨架（build+单测+推镜像）</t>
         </is>
       </c>
       <c r="F10" s="43" t="n"/>
@@ -2693,7 +2751,7 @@
       </c>
       <c r="E11" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 测试计划初稿（按 8 域组织：迁移/治理/生命周期/安全/检索/合规/连接器/权限）</t>
+          <t>• 🤖 测试计划初稿（8 域）</t>
         </is>
       </c>
       <c r="F11" s="42" t="inlineStr">
@@ -2701,11 +2759,7 @@
           <t>测试计划；架构图×2</t>
         </is>
       </c>
-      <c r="G11" s="29" t="inlineStr">
-        <is>
-          <t>BA 的 BRD 范围</t>
-        </is>
-      </c>
+      <c r="G11" s="29" t="inlineStr"/>
     </row>
     <row r="12" ht="22" customHeight="1" s="18">
       <c r="A12" s="43" t="n"/>
@@ -2714,7 +2768,7 @@
       <c r="D12" s="48" t="n"/>
       <c r="E12" s="41" t="inlineStr">
         <is>
-          <t>• 架构图初稿：上下文图 + 容器图</t>
+          <t>• 架构图初稿：上下文+容器图</t>
         </is>
       </c>
       <c r="F12" s="43" t="n"/>
@@ -2727,7 +2781,7 @@
       <c r="D13" s="48" t="n"/>
       <c r="E13" s="41" t="inlineStr">
         <is>
-          <t>• 文档模板 4 套定稿</t>
+          <t>• 文档模板 4 套</t>
         </is>
       </c>
       <c r="F13" s="43" t="n"/>
@@ -2756,7 +2810,7 @@
       </c>
       <c r="E14" s="41" t="inlineStr">
         <is>
-          <t>• BRD 评审 → 定稿签字</t>
+          <t>• BRD 评审→定稿签字</t>
         </is>
       </c>
       <c r="F14" s="42" t="inlineStr">
@@ -2777,7 +2831,7 @@
       <c r="D15" s="44" t="n"/>
       <c r="E15" s="41" t="inlineStr">
         <is>
-          <t>• CC 首批 50 张热表清单确认（业务方勾选）</t>
+          <t>• CC 首批 50 张热表清单确认</t>
         </is>
       </c>
       <c r="F15" s="43" t="n"/>
@@ -2806,7 +2860,7 @@
       </c>
       <c r="E16" s="41" t="inlineStr">
         <is>
-          <t>• 平台交付资源验收 + UC 初始化（arch_cc + GRANT 模板 + SP）</t>
+          <t>• 平台资源验收 + UC 初始化（arch_cc+GRANT+SP）</t>
         </is>
       </c>
       <c r="F16" s="42" t="inlineStr">
@@ -2820,14 +2874,14 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" s="18">
+    <row r="17" ht="22" customHeight="1" s="18">
       <c r="A17" s="43" t="n"/>
       <c r="B17" s="43" t="n"/>
       <c r="C17" s="43" t="n"/>
       <c r="D17" s="46" t="n"/>
       <c r="E17" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 SeaTunnel PoC：抽样 10 表 → RAW → SQL Warehouse 可查</t>
+          <t>• 🤖 SeaTunnel PoC：抽样 10 表端到端</t>
         </is>
       </c>
       <c r="F17" s="43" t="n"/>
@@ -2840,7 +2894,7 @@
       <c r="D18" s="46" t="n"/>
       <c r="E18" s="41" t="inlineStr">
         <is>
-          <t>• 【01】50 表批量导入（分片/限速/断点）+ 配置生成器 v1</t>
+          <t>• 【01】50 表批量导入 + 配置生成器 v1</t>
         </is>
       </c>
       <c r="F18" s="43" t="n"/>
@@ -2869,7 +2923,7 @@
       </c>
       <c r="E19" s="41" t="inlineStr">
         <is>
-          <t>• 架构图完善：组件图 + 部署图</t>
+          <t>• 架构图完善：组件+部署图</t>
         </is>
       </c>
       <c r="F19" s="42" t="inlineStr">
@@ -2886,7 +2940,7 @@
       <c r="D20" s="48" t="n"/>
       <c r="E20" s="41" t="inlineStr">
         <is>
-          <t>• 【01】迁移对账测试设计（行数/校验和）</t>
+          <t>• 【01】对账测试设计</t>
         </is>
       </c>
       <c r="F20" s="43" t="n"/>
@@ -2932,7 +2986,7 @@
       <c r="D22" s="44" t="n"/>
       <c r="E22" s="41" t="inlineStr">
         <is>
-          <t>• 预览格式范围确认（图片/音频/视频）</t>
+          <t>• 预览格式范围确认</t>
         </is>
       </c>
       <c r="F22" s="43" t="n"/>
@@ -2961,7 +3015,7 @@
       </c>
       <c r="E23" s="41" t="inlineStr">
         <is>
-          <t>• 【08】RBAC CRUD + OIDC/JWT 鉴权 + 前端权限渲染（🤖 AI 生成）</t>
+          <t>• 🤖【08】RBAC CRUD + OIDC/JWT 鉴权 + 前端权限渲染</t>
         </is>
       </c>
       <c r="F23" s="42" t="inlineStr">
@@ -2978,7 +3032,7 @@
       <c r="D24" s="46" t="n"/>
       <c r="E24" s="41" t="inlineStr">
         <is>
-          <t>• 【05】配置化检索页（动态筛选/表格/分页）</t>
+          <t>• 🤖【05】配置化检索页（动态筛选/表格/分页）</t>
         </is>
       </c>
       <c r="F24" s="43" t="n"/>
@@ -2991,7 +3045,7 @@
       <c r="D25" s="46" t="n"/>
       <c r="E25" s="41" t="inlineStr">
         <is>
-          <t>• 【06】审计埋点 v1 + 安全门禁①②进 CI</t>
+          <t>• 【06】审计埋点 v1</t>
         </is>
       </c>
       <c r="F25" s="43" t="n"/>
@@ -3020,7 +3074,7 @@
       </c>
       <c r="E26" s="41" t="inlineStr">
         <is>
-          <t>• 单测框架 + 覆盖率门禁 &gt;70% 进 CI</t>
+          <t>• 单测框架+覆盖率门禁 &gt;70%</t>
         </is>
       </c>
       <c r="F26" s="42" t="inlineStr">
@@ -3041,7 +3095,7 @@
       <c r="D27" s="48" t="n"/>
       <c r="E27" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 API 集成测试 10 场景（AI 生成用例）</t>
+          <t>• 🤖 API 集成测试 10 场景</t>
         </is>
       </c>
       <c r="F27" s="43" t="n"/>
@@ -3070,12 +3124,12 @@
       </c>
       <c r="E28" s="41" t="inlineStr">
         <is>
-          <t>• R1 核心场景验收（检索/预览/导出/权限三态对照用户故事）</t>
+          <t>• R1 功能验收（检索/预览/导出/权限三态）</t>
         </is>
       </c>
       <c r="F28" s="42" t="inlineStr">
         <is>
-          <t>R1 验收记录</t>
+          <t>R1 功能验收记录</t>
         </is>
       </c>
       <c r="G28" s="29" t="inlineStr"/>
@@ -3093,7 +3147,7 @@
       <c r="F29" s="43" t="n"/>
       <c r="G29" s="43" t="n"/>
     </row>
-    <row r="30" ht="30" customHeight="1" s="18">
+    <row r="30" ht="22" customHeight="1" s="18">
       <c r="A30" s="38" t="inlineStr">
         <is>
           <t>R1</t>
@@ -3116,12 +3170,12 @@
       </c>
       <c r="E30" s="41" t="inlineStr">
         <is>
-          <t>• 【08】UC GRANT 落地 + 掩码函数（aes_encrypt+COLUMN MASK）+ 权限三态联调</t>
+          <t>• 【08】UC GRANT+掩码函数+权限三态联调</t>
         </is>
       </c>
       <c r="F30" s="42" t="inlineStr">
         <is>
-          <t>权限三态通过；预览/导出可用</t>
+          <t>★ R1 功能全部 Done</t>
         </is>
       </c>
       <c r="G30" s="29" t="inlineStr"/>
@@ -3133,7 +3187,7 @@
       <c r="D31" s="46" t="n"/>
       <c r="E31" s="41" t="inlineStr">
         <is>
-          <t>• 【05】SERVE 热表物化 + 预览（SAS）+ 导出</t>
+          <t>• 【05】SERVE 物化+预览（SAS）+导出</t>
         </is>
       </c>
       <c r="F31" s="43" t="n"/>
@@ -3146,7 +3200,7 @@
       <c r="D32" s="46" t="n"/>
       <c r="E32" s="41" t="inlineStr">
         <is>
-          <t>• 安全修复 High 清零</t>
+          <t>• 安全门禁①②上线 + High 清零</t>
         </is>
       </c>
       <c r="F32" s="43" t="n"/>
@@ -3175,7 +3229,7 @@
       </c>
       <c r="E33" s="41" t="inlineStr">
         <is>
-          <t>• 功能测试执行 + Bug 跟踪</t>
+          <t>• 功能测试执行+Bug 跟踪</t>
         </is>
       </c>
       <c r="F33" s="42" t="inlineStr">
@@ -3192,7 +3246,7 @@
       <c r="D34" s="48" t="n"/>
       <c r="E34" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 安全测试①：注入/XSS/越权用例</t>
+          <t>• 🤖 安全测试①：注入/XSS/越权</t>
         </is>
       </c>
       <c r="F34" s="43" t="n"/>
@@ -3219,7 +3273,7 @@
       </c>
       <c r="B36" s="39" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C36" s="26" t="inlineStr">
@@ -3234,17 +3288,17 @@
       </c>
       <c r="E36" s="41" t="inlineStr">
         <is>
-          <t>• UAT #1 预演主持（Staging：检索/权限/审计场景）</t>
+          <t>• UAT #1 脚本定稿</t>
         </is>
       </c>
       <c r="F36" s="42" t="inlineStr">
         <is>
-          <t>预演完成</t>
+          <t>UAT #1 脚本</t>
         </is>
       </c>
       <c r="G36" s="29" t="inlineStr">
         <is>
-          <t>业务方预演排期</t>
+          <t>业务方排期</t>
         </is>
       </c>
     </row>
@@ -3255,13 +3309,13 @@
       <c r="D37" s="44" t="n"/>
       <c r="E37" s="41" t="inlineStr">
         <is>
-          <t>• 预演反馈分类与裁决</t>
+          <t>• 预演协调（业务方排期）</t>
         </is>
       </c>
       <c r="F37" s="43" t="n"/>
       <c r="G37" s="43" t="n"/>
     </row>
-    <row r="38" ht="22" customHeight="1" s="18">
+    <row r="38" ht="30" customHeight="1" s="18">
       <c r="A38" s="38" t="inlineStr">
         <is>
           <t>R1</t>
@@ -3269,7 +3323,7 @@
       </c>
       <c r="B38" s="39" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C38" s="26" t="inlineStr">
@@ -3284,17 +3338,17 @@
       </c>
       <c r="E38" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 R1 发布包（Helm 生产 values + UC 生产脚本）+ 回退演练</t>
+          <t>• 【DevOps】CD 流水线完善：Helm 多环境（Dev/Staging/Prod）+ Environments 审批流</t>
         </is>
       </c>
       <c r="F38" s="42" t="inlineStr">
         <is>
-          <t>发布包就绪；预跑完成</t>
+          <t>CD 就绪；发布包 v1</t>
         </is>
       </c>
       <c r="G38" s="29" t="inlineStr">
         <is>
-          <t>生产窗口审批</t>
+          <t>生产环境权限</t>
         </is>
       </c>
     </row>
@@ -3305,7 +3359,7 @@
       <c r="D39" s="46" t="n"/>
       <c r="E39" s="41" t="inlineStr">
         <is>
-          <t>• CC 生产迁移预跑（50 表→Staging）+ Runbook</t>
+          <t>• 【DevOps】安全门禁③④上线（gitleaks+Trivy，四道全开）</t>
         </is>
       </c>
       <c r="F39" s="43" t="n"/>
@@ -3318,7 +3372,7 @@
       <c r="D40" s="46" t="n"/>
       <c r="E40" s="41" t="inlineStr">
         <is>
-          <t>• 功能收口：性能优化（P95&lt;5s）+ 遗留清零 + 监控告警就绪</t>
+          <t>• 🤖 生产发布包（Helm 生产 values+UC 生产脚本）</t>
         </is>
       </c>
       <c r="F40" s="43" t="n"/>
@@ -3332,7 +3386,7 @@
       </c>
       <c r="B41" s="39" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C41" s="26" t="inlineStr">
@@ -3347,19 +3401,15 @@
       </c>
       <c r="E41" s="41" t="inlineStr">
         <is>
-          <t>• R1 文档冲刺：用户手册 50% + 运维手册 40%</t>
+          <t>• R1 文档冲刺：用户手册 60%</t>
         </is>
       </c>
       <c r="F41" s="42" t="inlineStr">
         <is>
-          <t>★ 就绪检查 100%</t>
-        </is>
-      </c>
-      <c r="G41" s="29" t="inlineStr">
-        <is>
-          <t>各角色材料</t>
-        </is>
-      </c>
+          <t>文档 60%</t>
+        </is>
+      </c>
+      <c r="G41" s="29" t="inlineStr"/>
     </row>
     <row r="42" ht="22" customHeight="1" s="18">
       <c r="A42" s="43" t="n"/>
@@ -3368,142 +3418,166 @@
       <c r="D42" s="48" t="n"/>
       <c r="E42" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 上线 Checklist v1 + UAT #1 脚本定稿</t>
+          <t>• 运维手册初稿（部署/监控部分）</t>
         </is>
       </c>
       <c r="F42" s="43" t="n"/>
       <c r="G42" s="43" t="n"/>
     </row>
     <row r="43" ht="22" customHeight="1" s="18">
-      <c r="A43" s="43" t="n"/>
-      <c r="B43" s="43" t="n"/>
-      <c r="C43" s="43" t="n"/>
-      <c r="D43" s="48" t="n"/>
+      <c r="A43" s="38" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B43" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C43" s="26" t="inlineStr">
+        <is>
+          <t>W6</t>
+        </is>
+      </c>
+      <c r="D43" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
+        </is>
+      </c>
       <c r="E43" s="41" t="inlineStr">
         <is>
-          <t>• W5 末就绪检查组织（发布包/预演/回退/预跑）</t>
-        </is>
-      </c>
-      <c r="F43" s="43" t="n"/>
-      <c r="G43" s="43" t="n"/>
+          <t>• UAT #1 预演主持（Staging：检索/权限/审计）</t>
+        </is>
+      </c>
+      <c r="F43" s="42" t="inlineStr">
+        <is>
+          <t>预演完成</t>
+        </is>
+      </c>
+      <c r="G43" s="29" t="inlineStr"/>
     </row>
     <row r="44" ht="22" customHeight="1" s="18">
-      <c r="A44" s="38" t="inlineStr">
+      <c r="A44" s="43" t="n"/>
+      <c r="B44" s="43" t="n"/>
+      <c r="C44" s="43" t="n"/>
+      <c r="D44" s="44" t="n"/>
+      <c r="E44" s="41" t="inlineStr">
+        <is>
+          <t>• 预演反馈裁决</t>
+        </is>
+      </c>
+      <c r="F44" s="43" t="n"/>
+      <c r="G44" s="43" t="n"/>
+    </row>
+    <row r="45" ht="22" customHeight="1" s="18">
+      <c r="A45" s="38" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B44" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="C44" s="26" t="inlineStr">
+      <c r="B45" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C45" s="26" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="D44" s="40" t="inlineStr">
-        <is>
-          <t>BA·Mandy</t>
-        </is>
-      </c>
-      <c r="E44" s="41" t="inlineStr">
-        <is>
-          <t>• Go/No-Go #1 决策参与</t>
-        </is>
-      </c>
-      <c r="F44" s="42" t="inlineStr">
-        <is>
-          <t>★ UAT #1 签字</t>
-        </is>
-      </c>
-      <c r="G44" s="29" t="inlineStr">
-        <is>
-          <t>UAT 业务方时间</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="22" customHeight="1" s="18">
-      <c r="A45" s="43" t="n"/>
-      <c r="B45" s="43" t="n"/>
-      <c r="C45" s="43" t="n"/>
-      <c r="D45" s="44" t="n"/>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
+        </is>
+      </c>
       <c r="E45" s="41" t="inlineStr">
         <is>
-          <t>• UAT #1 正式主持（签字）</t>
-        </is>
-      </c>
-      <c r="F45" s="43" t="n"/>
-      <c r="G45" s="43" t="n"/>
+          <t>• 回退预案演练（发布回滚+UC 配置回滚）</t>
+        </is>
+      </c>
+      <c r="F45" s="42" t="inlineStr">
+        <is>
+          <t>回退演练过；预跑完成</t>
+        </is>
+      </c>
+      <c r="G45" s="29" t="inlineStr">
+        <is>
+          <t>生产窗口审批</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="22" customHeight="1" s="18">
       <c r="A46" s="43" t="n"/>
       <c r="B46" s="43" t="n"/>
       <c r="C46" s="43" t="n"/>
-      <c r="D46" s="44" t="n"/>
+      <c r="D46" s="46" t="n"/>
       <c r="E46" s="41" t="inlineStr">
         <is>
-          <t>• 上线后用户反馈分诊</t>
+          <t>• 监控告警就绪（App Insights+Dashboard）</t>
         </is>
       </c>
       <c r="F46" s="43" t="n"/>
       <c r="G46" s="43" t="n"/>
     </row>
     <row r="47" ht="22" customHeight="1" s="18">
-      <c r="A47" s="38" t="inlineStr">
+      <c r="A47" s="43" t="n"/>
+      <c r="B47" s="43" t="n"/>
+      <c r="C47" s="43" t="n"/>
+      <c r="D47" s="46" t="n"/>
+      <c r="E47" s="41" t="inlineStr">
+        <is>
+          <t>• CC 迁移预跑（50 表→Staging）+ Runbook</t>
+        </is>
+      </c>
+      <c r="F47" s="43" t="n"/>
+      <c r="G47" s="43" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1" s="18">
+      <c r="A48" s="38" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B47" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 2</t>
-        </is>
-      </c>
-      <c r="C47" s="26" t="inlineStr">
+      <c r="B48" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 3</t>
+        </is>
+      </c>
+      <c r="C48" s="26" t="inlineStr">
         <is>
           <t>W6</t>
         </is>
       </c>
-      <c r="D47" s="45" t="inlineStr">
-        <is>
-          <t>DEV·Wade</t>
-        </is>
-      </c>
-      <c r="E47" s="41" t="inlineStr">
-        <is>
-          <t>• 生产发布执行（就绪包一键发布+审批）</t>
-        </is>
-      </c>
-      <c r="F47" s="42" t="inlineStr">
-        <is>
-          <t>★ Go-Live #1</t>
-        </is>
-      </c>
-      <c r="G47" s="29" t="inlineStr"/>
-    </row>
-    <row r="48" ht="22" customHeight="1" s="18">
-      <c r="A48" s="43" t="n"/>
-      <c r="B48" s="43" t="n"/>
-      <c r="C48" s="43" t="n"/>
-      <c r="D48" s="46" t="n"/>
+      <c r="D48" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="E48" s="41" t="inlineStr">
         <is>
-          <t>• CC 50 表生产迁移+对账</t>
-        </is>
-      </c>
-      <c r="F48" s="43" t="n"/>
-      <c r="G48" s="43" t="n"/>
+          <t>• 上线 Checklist v1</t>
+        </is>
+      </c>
+      <c r="F48" s="42" t="inlineStr">
+        <is>
+          <t>★ R1 就绪检查 100%</t>
+        </is>
+      </c>
+      <c r="G48" s="29" t="inlineStr">
+        <is>
+          <t>各角色材料</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="22" customHeight="1" s="18">
       <c r="A49" s="43" t="n"/>
       <c r="B49" s="43" t="n"/>
       <c r="C49" s="43" t="n"/>
-      <c r="D49" s="46" t="n"/>
+      <c r="D49" s="48" t="n"/>
       <c r="E49" s="41" t="inlineStr">
         <is>
-          <t>• P1 当日清 + 48h 值守</t>
+          <t>• W6 末就绪检查组织（CD/发布包/预演/回退/预跑）</t>
         </is>
       </c>
       <c r="F49" s="43" t="n"/>
@@ -3517,32 +3591,32 @@
       </c>
       <c r="B50" s="39" t="inlineStr">
         <is>
-          <t>Sprint 2</t>
+          <t>Sprint 3</t>
         </is>
       </c>
       <c r="C50" s="26" t="inlineStr">
         <is>
-          <t>W6</t>
-        </is>
-      </c>
-      <c r="D50" s="47" t="inlineStr">
-        <is>
-          <t>QA</t>
+          <t>W7</t>
+        </is>
+      </c>
+      <c r="D50" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
         </is>
       </c>
       <c r="E50" s="41" t="inlineStr">
         <is>
-          <t>• 上线执行记录（Checklist 勾选）</t>
+          <t>• Go/No-Go #1 决策参与</t>
         </is>
       </c>
       <c r="F50" s="42" t="inlineStr">
         <is>
-          <t>★ Release 1 交付</t>
+          <t>★ UAT #1 签字</t>
         </is>
       </c>
       <c r="G50" s="29" t="inlineStr">
         <is>
-          <t>审批受理</t>
+          <t>UAT 业务方时间</t>
         </is>
       </c>
     </row>
@@ -3550,10 +3624,10 @@
       <c r="A51" s="43" t="n"/>
       <c r="B51" s="43" t="n"/>
       <c r="C51" s="43" t="n"/>
-      <c r="D51" s="48" t="n"/>
+      <c r="D51" s="44" t="n"/>
       <c r="E51" s="41" t="inlineStr">
         <is>
-          <t>• R1 审批材料提交</t>
+          <t>• UAT #1 正式主持（签字）</t>
         </is>
       </c>
       <c r="F51" s="43" t="n"/>
@@ -3563,19 +3637,19 @@
       <c r="A52" s="43" t="n"/>
       <c r="B52" s="43" t="n"/>
       <c r="C52" s="43" t="n"/>
-      <c r="D52" s="48" t="n"/>
+      <c r="D52" s="44" t="n"/>
       <c r="E52" s="41" t="inlineStr">
         <is>
-          <t>• 48h 值守轮值</t>
+          <t>• 上线后反馈分诊</t>
         </is>
       </c>
       <c r="F52" s="43" t="n"/>
       <c r="G52" s="43" t="n"/>
     </row>
     <row r="53" ht="22" customHeight="1" s="18">
-      <c r="A53" s="49" t="inlineStr">
-        <is>
-          <t>R2</t>
+      <c r="A53" s="38" t="inlineStr">
+        <is>
+          <t>R1</t>
         </is>
       </c>
       <c r="B53" s="39" t="inlineStr">
@@ -3588,177 +3662,161 @@
           <t>W7</t>
         </is>
       </c>
-      <c r="D53" s="40" t="inlineStr">
-        <is>
-          <t>BA·Mandy</t>
+      <c r="D53" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
         </is>
       </c>
       <c r="E53" s="41" t="inlineStr">
         <is>
-          <t>• 【02】增量频率与冷数据标准确认</t>
+          <t>• 生产发布执行（就绪包+审批）</t>
         </is>
       </c>
       <c r="F53" s="42" t="inlineStr">
         <is>
-          <t>R2 需求就绪</t>
-        </is>
-      </c>
-      <c r="G53" s="29" t="inlineStr">
-        <is>
-          <t>法务配合</t>
-        </is>
-      </c>
+          <t>★ Go-Live #1</t>
+        </is>
+      </c>
+      <c r="G53" s="29" t="inlineStr"/>
     </row>
     <row r="54" ht="22" customHeight="1" s="18">
       <c r="A54" s="43" t="n"/>
       <c r="B54" s="43" t="n"/>
       <c r="C54" s="43" t="n"/>
-      <c r="D54" s="44" t="n"/>
+      <c r="D54" s="46" t="n"/>
       <c r="E54" s="41" t="inlineStr">
         <is>
-          <t>• 【03】Legal Hold 触发条件定稿（法务）</t>
+          <t>• CC 50 表生产迁移+对账</t>
         </is>
       </c>
       <c r="F54" s="43" t="n"/>
       <c r="G54" s="43" t="n"/>
     </row>
     <row r="55" ht="22" customHeight="1" s="18">
-      <c r="A55" s="49" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B55" s="39" t="inlineStr">
+      <c r="A55" s="43" t="n"/>
+      <c r="B55" s="43" t="n"/>
+      <c r="C55" s="43" t="n"/>
+      <c r="D55" s="46" t="n"/>
+      <c r="E55" s="41" t="inlineStr">
+        <is>
+          <t>• P1 当日清+48h 值守</t>
+        </is>
+      </c>
+      <c r="F55" s="43" t="n"/>
+      <c r="G55" s="43" t="n"/>
+    </row>
+    <row r="56" ht="22" customHeight="1" s="18">
+      <c r="A56" s="38" t="inlineStr">
+        <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B56" s="39" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="C55" s="26" t="inlineStr">
+      <c r="C56" s="26" t="inlineStr">
         <is>
           <t>W7</t>
         </is>
       </c>
-      <c r="D55" s="45" t="inlineStr">
-        <is>
-          <t>DEV·Wade</t>
-        </is>
-      </c>
-      <c r="E55" s="41" t="inlineStr">
-        <is>
-          <t>• 【03】处置引擎（扫描→DROP PARTITION→VACUUM）</t>
-        </is>
-      </c>
-      <c r="F55" s="42" t="inlineStr">
-        <is>
-          <t>处置引擎可跑；加密生效</t>
-        </is>
-      </c>
-      <c r="G55" s="29" t="inlineStr"/>
-    </row>
-    <row r="56" ht="22" customHeight="1" s="18">
-      <c r="A56" s="43" t="n"/>
-      <c r="B56" s="43" t="n"/>
-      <c r="C56" s="43" t="n"/>
-      <c r="D56" s="46" t="n"/>
+      <c r="D56" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="E56" s="41" t="inlineStr">
         <is>
-          <t>• 【04】加密体系（CMK+字段级+密钥轮转）</t>
-        </is>
-      </c>
-      <c r="F56" s="43" t="n"/>
-      <c r="G56" s="43" t="n"/>
+          <t>• 上线执行记录</t>
+        </is>
+      </c>
+      <c r="F56" s="42" t="inlineStr">
+        <is>
+          <t>★ Release 1 交付</t>
+        </is>
+      </c>
+      <c r="G56" s="29" t="inlineStr">
+        <is>
+          <t>审批受理</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="22" customHeight="1" s="18">
       <c r="A57" s="43" t="n"/>
       <c r="B57" s="43" t="n"/>
       <c r="C57" s="43" t="n"/>
-      <c r="D57" s="46" t="n"/>
+      <c r="D57" s="48" t="n"/>
       <c r="E57" s="41" t="inlineStr">
         <is>
-          <t>• 【02】增量接入（watermark）+ 冷数据自动转冷</t>
+          <t>• R1 审批材料提交</t>
         </is>
       </c>
       <c r="F57" s="43" t="n"/>
       <c r="G57" s="43" t="n"/>
     </row>
     <row r="58" ht="22" customHeight="1" s="18">
-      <c r="A58" s="49" t="inlineStr">
+      <c r="A58" s="43" t="n"/>
+      <c r="B58" s="43" t="n"/>
+      <c r="C58" s="43" t="n"/>
+      <c r="D58" s="48" t="n"/>
+      <c r="E58" s="41" t="inlineStr">
+        <is>
+          <t>• 48h 值守轮值</t>
+        </is>
+      </c>
+      <c r="F58" s="43" t="n"/>
+      <c r="G58" s="43" t="n"/>
+    </row>
+    <row r="59" ht="22" customHeight="1" s="18">
+      <c r="A59" s="49" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B58" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="C58" s="26" t="inlineStr">
-        <is>
-          <t>W7</t>
-        </is>
-      </c>
-      <c r="D58" s="47" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="E58" s="41" t="inlineStr">
-        <is>
-          <t>• 功能用例扩充（处置/Hold/增量/脱敏）</t>
-        </is>
-      </c>
-      <c r="F58" s="42" t="inlineStr">
-        <is>
-          <t>用例扩充</t>
-        </is>
-      </c>
-      <c r="G58" s="29" t="inlineStr"/>
-    </row>
-    <row r="59" ht="22" customHeight="1" s="18">
-      <c r="A59" s="43" t="n"/>
-      <c r="B59" s="43" t="n"/>
-      <c r="C59" s="43" t="n"/>
-      <c r="D59" s="48" t="n"/>
+      <c r="B59" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C59" s="26" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="D59" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
+        </is>
+      </c>
       <c r="E59" s="41" t="inlineStr">
         <is>
-          <t>• R1 上线后回归监控 + 文档推进（手册 60%）</t>
-        </is>
-      </c>
-      <c r="F59" s="43" t="n"/>
-      <c r="G59" s="43" t="n"/>
+          <t>• 【02】增量频率与冷数据标准确认</t>
+        </is>
+      </c>
+      <c r="F59" s="42" t="inlineStr">
+        <is>
+          <t>R2 需求就绪</t>
+        </is>
+      </c>
+      <c r="G59" s="29" t="inlineStr">
+        <is>
+          <t>法务配合</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="22" customHeight="1" s="18">
-      <c r="A60" s="49" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B60" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="C60" s="26" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="D60" s="40" t="inlineStr">
-        <is>
-          <t>BA·Mandy</t>
-        </is>
-      </c>
+      <c r="A60" s="43" t="n"/>
+      <c r="B60" s="43" t="n"/>
+      <c r="C60" s="43" t="n"/>
+      <c r="D60" s="44" t="n"/>
       <c r="E60" s="41" t="inlineStr">
         <is>
-          <t>• 验收处置全链路（对照合规要求）</t>
-        </is>
-      </c>
-      <c r="F60" s="42" t="inlineStr">
-        <is>
-          <t>处置验收</t>
-        </is>
-      </c>
-      <c r="G60" s="29" t="inlineStr"/>
+          <t>• 【03】Legal Hold 触发条件定稿（法务）</t>
+        </is>
+      </c>
+      <c r="F60" s="43" t="n"/>
+      <c r="G60" s="43" t="n"/>
     </row>
     <row r="61" ht="22" customHeight="1" s="18">
       <c r="A61" s="49" t="inlineStr">
@@ -3768,7 +3826,7 @@
       </c>
       <c r="B61" s="39" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="C61" s="26" t="inlineStr">
@@ -3783,12 +3841,12 @@
       </c>
       <c r="E61" s="41" t="inlineStr">
         <is>
-          <t>• 【03】Legal Hold（Hold/Release+豁免+留痕）+ 归档模型管理</t>
+          <t>• 【03】处置引擎（扫描→DROP PARTITION→VACUUM）</t>
         </is>
       </c>
       <c r="F61" s="42" t="inlineStr">
         <is>
-          <t>Hold 可用；分层生效</t>
+          <t>处置引擎可跑；加密生效</t>
         </is>
       </c>
       <c r="G61" s="29" t="inlineStr"/>
@@ -3800,7 +3858,7 @@
       <c r="D62" s="46" t="n"/>
       <c r="E62" s="41" t="inlineStr">
         <is>
-          <t>• 【04】境内驻留核查（区域+出口流量）</t>
+          <t>• 【04】加密体系（CMK+字段级+轮转）</t>
         </is>
       </c>
       <c r="F62" s="43" t="n"/>
@@ -3813,70 +3871,90 @@
       <c r="D63" s="46" t="n"/>
       <c r="E63" s="41" t="inlineStr">
         <is>
-          <t>• 【04】ADLS 分层+生命周期+Compaction</t>
+          <t>• 【02】增量接入（watermark）</t>
         </is>
       </c>
       <c r="F63" s="43" t="n"/>
       <c r="G63" s="43" t="n"/>
     </row>
     <row r="64" ht="22" customHeight="1" s="18">
-      <c r="A64" s="43" t="n"/>
-      <c r="B64" s="43" t="n"/>
-      <c r="C64" s="43" t="n"/>
-      <c r="D64" s="46" t="n"/>
+      <c r="A64" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B64" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C64" s="26" t="inlineStr">
+        <is>
+          <t>W8</t>
+        </is>
+      </c>
+      <c r="D64" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="E64" s="41" t="inlineStr">
         <is>
-          <t>• 【07】连接器模板库（MySQL+文件源）</t>
-        </is>
-      </c>
-      <c r="F64" s="43" t="n"/>
-      <c r="G64" s="43" t="n"/>
+          <t>• 功能用例扩充（处置/Hold/增量/脱敏）</t>
+        </is>
+      </c>
+      <c r="F64" s="42" t="inlineStr">
+        <is>
+          <t>用例扩充</t>
+        </is>
+      </c>
+      <c r="G64" s="29" t="inlineStr"/>
     </row>
     <row r="65" ht="22" customHeight="1" s="18">
-      <c r="A65" s="49" t="inlineStr">
+      <c r="A65" s="43" t="n"/>
+      <c r="B65" s="43" t="n"/>
+      <c r="C65" s="43" t="n"/>
+      <c r="D65" s="48" t="n"/>
+      <c r="E65" s="41" t="inlineStr">
+        <is>
+          <t>• R1 生产回归监控</t>
+        </is>
+      </c>
+      <c r="F65" s="43" t="n"/>
+      <c r="G65" s="43" t="n"/>
+    </row>
+    <row r="66" ht="22" customHeight="1" s="18">
+      <c r="A66" s="49" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B65" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="C65" s="26" t="inlineStr">
-        <is>
-          <t>W8</t>
-        </is>
-      </c>
-      <c r="D65" s="47" t="inlineStr">
-        <is>
-          <t>QA</t>
-        </is>
-      </c>
-      <c r="E65" s="41" t="inlineStr">
-        <is>
-          <t>• 【03】处置全链路 E2E：1 天保留期→到期→Hold→处置→审计</t>
-        </is>
-      </c>
-      <c r="F65" s="42" t="inlineStr">
-        <is>
-          <t>处置 E2E 通过</t>
-        </is>
-      </c>
-      <c r="G65" s="29" t="inlineStr"/>
-    </row>
-    <row r="66" ht="22" customHeight="1" s="18">
-      <c r="A66" s="43" t="n"/>
-      <c r="B66" s="43" t="n"/>
-      <c r="C66" s="43" t="n"/>
-      <c r="D66" s="48" t="n"/>
+      <c r="B66" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C66" s="26" t="inlineStr">
+        <is>
+          <t>W9</t>
+        </is>
+      </c>
+      <c r="D66" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
+        </is>
+      </c>
       <c r="E66" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 安全测试②：掩码旁路/越权用例</t>
-        </is>
-      </c>
-      <c r="F66" s="43" t="n"/>
-      <c r="G66" s="43" t="n"/>
+          <t>• 验收处置全链路（对照合规）</t>
+        </is>
+      </c>
+      <c r="F66" s="42" t="inlineStr">
+        <is>
+          <t>处置验收</t>
+        </is>
+      </c>
+      <c r="G66" s="29" t="inlineStr"/>
     </row>
     <row r="67" ht="22" customHeight="1" s="18">
       <c r="A67" s="49" t="inlineStr">
@@ -3886,7 +3964,7 @@
       </c>
       <c r="B67" s="39" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 4</t>
         </is>
       </c>
       <c r="C67" s="26" t="inlineStr">
@@ -3894,19 +3972,19 @@
           <t>W9</t>
         </is>
       </c>
-      <c r="D67" s="40" t="inlineStr">
-        <is>
-          <t>BA·Mandy</t>
+      <c r="D67" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
         </is>
       </c>
       <c r="E67" s="41" t="inlineStr">
         <is>
-          <t>• 合规报表口径与法务对齐</t>
+          <t>• 【03】Legal Hold+归档模型+处置界面</t>
         </is>
       </c>
       <c r="F67" s="42" t="inlineStr">
         <is>
-          <t>口径确认；范围签字</t>
+          <t>Hold 可用；分层生效</t>
         </is>
       </c>
       <c r="G67" s="29" t="inlineStr"/>
@@ -3915,73 +3993,69 @@
       <c r="A68" s="43" t="n"/>
       <c r="B68" s="43" t="n"/>
       <c r="C68" s="43" t="n"/>
-      <c r="D68" s="44" t="n"/>
+      <c r="D68" s="46" t="n"/>
       <c r="E68" s="41" t="inlineStr">
         <is>
-          <t>• CC 全量迁移范围最终确认（签字）</t>
+          <t>• 【04】驻留核查+ADLS 分层+Compaction</t>
         </is>
       </c>
       <c r="F68" s="43" t="n"/>
       <c r="G68" s="43" t="n"/>
     </row>
     <row r="69" ht="22" customHeight="1" s="18">
-      <c r="A69" s="49" t="inlineStr">
+      <c r="A69" s="43" t="n"/>
+      <c r="B69" s="43" t="n"/>
+      <c r="C69" s="43" t="n"/>
+      <c r="D69" s="46" t="n"/>
+      <c r="E69" s="41" t="inlineStr">
+        <is>
+          <t>• 【07】连接器模板库（MySQL+文件源）</t>
+        </is>
+      </c>
+      <c r="F69" s="43" t="n"/>
+      <c r="G69" s="43" t="n"/>
+    </row>
+    <row r="70" ht="22" customHeight="1" s="18">
+      <c r="A70" s="49" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B69" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 3</t>
-        </is>
-      </c>
-      <c r="C69" s="26" t="inlineStr">
+      <c r="B70" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 4</t>
+        </is>
+      </c>
+      <c r="C70" s="26" t="inlineStr">
         <is>
           <t>W9</t>
         </is>
       </c>
-      <c r="D69" s="45" t="inlineStr">
-        <is>
-          <t>DEV·Wade</t>
-        </is>
-      </c>
-      <c r="E69" s="41" t="inlineStr">
-        <is>
-          <t>• 【08】行级隔离验证（越权全拦）</t>
-        </is>
-      </c>
-      <c r="F69" s="42" t="inlineStr">
-        <is>
-          <t>全量启动；越权拦截</t>
-        </is>
-      </c>
-      <c r="G69" s="29" t="inlineStr">
-        <is>
-          <t>CC 数据量实测</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="22" customHeight="1" s="18">
-      <c r="A70" s="43" t="n"/>
-      <c r="B70" s="43" t="n"/>
-      <c r="C70" s="43" t="n"/>
-      <c r="D70" s="46" t="n"/>
+      <c r="D70" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
       <c r="E70" s="41" t="inlineStr">
         <is>
-          <t>• 【01】CC 全量 1253 表分批迁移启动（600~800 有效表）</t>
-        </is>
-      </c>
-      <c r="F70" s="43" t="n"/>
-      <c r="G70" s="43" t="n"/>
+          <t>• 【03】处置全链路 E2E（1 天保留期→到期→Hold→处置→审计）</t>
+        </is>
+      </c>
+      <c r="F70" s="42" t="inlineStr">
+        <is>
+          <t>处置 E2E 通过</t>
+        </is>
+      </c>
+      <c r="G70" s="29" t="inlineStr"/>
     </row>
     <row r="71" ht="22" customHeight="1" s="18">
       <c r="A71" s="43" t="n"/>
       <c r="B71" s="43" t="n"/>
       <c r="C71" s="43" t="n"/>
-      <c r="D71" s="46" t="n"/>
+      <c r="D71" s="48" t="n"/>
       <c r="E71" s="41" t="inlineStr">
         <is>
-          <t>• 【07】连接器运行监控与审计</t>
+          <t>• 🤖 安全测试②：掩码旁路/越权</t>
         </is>
       </c>
       <c r="F71" s="43" t="n"/>
@@ -3995,27 +4069,27 @@
       </c>
       <c r="B72" s="39" t="inlineStr">
         <is>
-          <t>Sprint 3</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="C72" s="26" t="inlineStr">
         <is>
-          <t>W9</t>
-        </is>
-      </c>
-      <c r="D72" s="47" t="inlineStr">
-        <is>
-          <t>QA</t>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="D72" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
         </is>
       </c>
       <c r="E72" s="41" t="inlineStr">
         <is>
-          <t>• 【07】连接器兼容性测试（SQL Server/MySQL 矩阵）</t>
+          <t>• 合规报表口径与法务对齐</t>
         </is>
       </c>
       <c r="F72" s="42" t="inlineStr">
         <is>
-          <t>兼容矩阵</t>
+          <t>口径确认；范围签字</t>
         </is>
       </c>
       <c r="G72" s="29" t="inlineStr"/>
@@ -4024,60 +4098,64 @@
       <c r="A73" s="43" t="n"/>
       <c r="B73" s="43" t="n"/>
       <c r="C73" s="43" t="n"/>
-      <c r="D73" s="48" t="n"/>
+      <c r="D73" s="44" t="n"/>
       <c r="E73" s="41" t="inlineStr">
         <is>
-          <t>• 【06】合规报表口径验证</t>
+          <t>• CC 全量范围最终确认（签字）</t>
         </is>
       </c>
       <c r="F73" s="43" t="n"/>
       <c r="G73" s="43" t="n"/>
     </row>
     <row r="74" ht="22" customHeight="1" s="18">
-      <c r="A74" s="43" t="n"/>
-      <c r="B74" s="43" t="n"/>
-      <c r="C74" s="43" t="n"/>
-      <c r="D74" s="48" t="n"/>
+      <c r="A74" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B74" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C74" s="26" t="inlineStr">
+        <is>
+          <t>W10</t>
+        </is>
+      </c>
+      <c r="D74" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
+        </is>
+      </c>
       <c r="E74" s="41" t="inlineStr">
         <is>
-          <t>• 用户手册 70% + 数据字典初稿</t>
-        </is>
-      </c>
-      <c r="F74" s="43" t="n"/>
-      <c r="G74" s="43" t="n"/>
+          <t>• 【01】CC 全量 1253 表分批迁移启动（600~800 有效表）</t>
+        </is>
+      </c>
+      <c r="F74" s="42" t="inlineStr">
+        <is>
+          <t>全量启动</t>
+        </is>
+      </c>
+      <c r="G74" s="29" t="inlineStr">
+        <is>
+          <t>CC 数据量实测</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="22" customHeight="1" s="18">
-      <c r="A75" s="49" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B75" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="C75" s="26" t="inlineStr">
-        <is>
-          <t>W10</t>
-        </is>
-      </c>
-      <c r="D75" s="40" t="inlineStr">
-        <is>
-          <t>BA·Mandy</t>
-        </is>
-      </c>
+      <c r="A75" s="43" t="n"/>
+      <c r="B75" s="43" t="n"/>
+      <c r="C75" s="43" t="n"/>
+      <c r="D75" s="46" t="n"/>
       <c r="E75" s="41" t="inlineStr">
         <is>
-          <t>• UAT #2 场景脚本定稿（处置/Hold/脱敏/报表）</t>
-        </is>
-      </c>
-      <c r="F75" s="42" t="inlineStr">
-        <is>
-          <t>UAT #2 脚本</t>
-        </is>
-      </c>
-      <c r="G75" s="29" t="inlineStr"/>
+          <t>• 【06】合规报表开发</t>
+        </is>
+      </c>
+      <c r="F75" s="43" t="n"/>
+      <c r="G75" s="43" t="n"/>
     </row>
     <row r="76" ht="22" customHeight="1" s="18">
       <c r="A76" s="49" t="inlineStr">
@@ -4087,7 +4165,7 @@
       </c>
       <c r="B76" s="39" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="C76" s="26" t="inlineStr">
@@ -4095,52 +4173,68 @@
           <t>W10</t>
         </is>
       </c>
-      <c r="D76" s="45" t="inlineStr">
-        <is>
-          <t>DEV·Wade</t>
+      <c r="D76" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
         </is>
       </c>
       <c r="E76" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 R2 发布包（增量/处置/加密/分层生产版）+ 回退演练</t>
+          <t>• 【07】连接器兼容性测试</t>
         </is>
       </c>
       <c r="F76" s="42" t="inlineStr">
         <is>
-          <t>R2 发布包就绪</t>
-        </is>
-      </c>
-      <c r="G76" s="29" t="inlineStr">
-        <is>
-          <t>生产窗口</t>
-        </is>
-      </c>
+          <t>兼容矩阵</t>
+        </is>
+      </c>
+      <c r="G76" s="29" t="inlineStr"/>
     </row>
     <row r="77" ht="22" customHeight="1" s="18">
       <c r="A77" s="43" t="n"/>
       <c r="B77" s="43" t="n"/>
       <c r="C77" s="43" t="n"/>
-      <c r="D77" s="46" t="n"/>
+      <c r="D77" s="48" t="n"/>
       <c r="E77" s="41" t="inlineStr">
         <is>
-          <t>• 安全评审材料（技术说明）</t>
+          <t>• 用户手册 70%+数据字典初稿</t>
         </is>
       </c>
       <c r="F77" s="43" t="n"/>
       <c r="G77" s="43" t="n"/>
     </row>
     <row r="78" ht="22" customHeight="1" s="18">
-      <c r="A78" s="43" t="n"/>
-      <c r="B78" s="43" t="n"/>
-      <c r="C78" s="43" t="n"/>
-      <c r="D78" s="46" t="n"/>
+      <c r="A78" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B78" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C78" s="26" t="inlineStr">
+        <is>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="D78" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
+        </is>
+      </c>
       <c r="E78" s="41" t="inlineStr">
         <is>
-          <t>• 【01】全量迁移继续 + 逐批对账 + 生产预跑</t>
-        </is>
-      </c>
-      <c r="F78" s="43" t="n"/>
-      <c r="G78" s="43" t="n"/>
+          <t>• UAT #2 场景脚本初稿</t>
+        </is>
+      </c>
+      <c r="F78" s="42" t="inlineStr">
+        <is>
+          <t>UAT #2 脚本初稿</t>
+        </is>
+      </c>
+      <c r="G78" s="29" t="inlineStr"/>
     </row>
     <row r="79" ht="22" customHeight="1" s="18">
       <c r="A79" s="49" t="inlineStr">
@@ -4150,27 +4244,27 @@
       </c>
       <c r="B79" s="39" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="C79" s="26" t="inlineStr">
         <is>
-          <t>W10</t>
-        </is>
-      </c>
-      <c r="D79" s="47" t="inlineStr">
-        <is>
-          <t>QA</t>
+          <t>W11</t>
+        </is>
+      </c>
+      <c r="D79" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
         </is>
       </c>
       <c r="E79" s="41" t="inlineStr">
         <is>
-          <t>• 文档冲刺：用户手册 85% + 运维手册 70% + 架构图更新</t>
+          <t>• 【01】全量迁移继续+逐批对账</t>
         </is>
       </c>
       <c r="F79" s="42" t="inlineStr">
         <is>
-          <t>文档 80%+</t>
+          <t>★ 全量对账 100%</t>
         </is>
       </c>
       <c r="G79" s="29" t="inlineStr"/>
@@ -4179,123 +4273,119 @@
       <c r="A80" s="43" t="n"/>
       <c r="B80" s="43" t="n"/>
       <c r="C80" s="43" t="n"/>
-      <c r="D80" s="48" t="n"/>
+      <c r="D80" s="46" t="n"/>
       <c r="E80" s="41" t="inlineStr">
         <is>
-          <t>• 🤖 审批材料起稿</t>
+          <t>• 【07】连接器运行监控+连接管理界面</t>
         </is>
       </c>
       <c r="F80" s="43" t="n"/>
       <c r="G80" s="43" t="n"/>
     </row>
     <row r="81" ht="22" customHeight="1" s="18">
-      <c r="A81" s="49" t="inlineStr">
+      <c r="A81" s="43" t="n"/>
+      <c r="B81" s="43" t="n"/>
+      <c r="C81" s="43" t="n"/>
+      <c r="D81" s="46" t="n"/>
+      <c r="E81" s="41" t="inlineStr">
+        <is>
+          <t>• 【08】行级隔离验证</t>
+        </is>
+      </c>
+      <c r="F81" s="43" t="n"/>
+      <c r="G81" s="43" t="n"/>
+    </row>
+    <row r="82" ht="22" customHeight="1" s="18">
+      <c r="A82" s="49" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B81" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="C81" s="26" t="inlineStr">
+      <c r="B82" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C82" s="26" t="inlineStr">
         <is>
           <t>W11</t>
         </is>
       </c>
-      <c r="D81" s="40" t="inlineStr">
+      <c r="D82" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="E82" s="41" t="inlineStr">
+        <is>
+          <t>• 【06】合规报表口径验证</t>
+        </is>
+      </c>
+      <c r="F82" s="42" t="inlineStr">
+        <is>
+          <t>报表验证过</t>
+        </is>
+      </c>
+      <c r="G82" s="29" t="inlineStr"/>
+    </row>
+    <row r="83" ht="22" customHeight="1" s="18">
+      <c r="A83" s="43" t="n"/>
+      <c r="B83" s="43" t="n"/>
+      <c r="C83" s="43" t="n"/>
+      <c r="D83" s="48" t="n"/>
+      <c r="E83" s="41" t="inlineStr">
+        <is>
+          <t>• 文档 80%（架构图更新+运维手册完善）</t>
+        </is>
+      </c>
+      <c r="F83" s="43" t="n"/>
+      <c r="G83" s="43" t="n"/>
+    </row>
+    <row r="84" ht="22" customHeight="1" s="18">
+      <c r="A84" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B84" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C84" s="26" t="inlineStr">
+        <is>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="D84" s="40" t="inlineStr">
         <is>
           <t>BA·Mandy</t>
         </is>
       </c>
-      <c r="E81" s="41" t="inlineStr">
-        <is>
-          <t>• UAT #2 预演主持（处置/Hold/脱敏/报表）</t>
-        </is>
-      </c>
-      <c r="F81" s="42" t="inlineStr">
-        <is>
-          <t>预演完成</t>
-        </is>
-      </c>
-      <c r="G81" s="29" t="inlineStr">
+      <c r="E84" s="41" t="inlineStr">
+        <is>
+          <t>• UAT #2 脚本定稿</t>
+        </is>
+      </c>
+      <c r="F84" s="42" t="inlineStr">
+        <is>
+          <t>UAT #2 脚本</t>
+        </is>
+      </c>
+      <c r="G84" s="29" t="inlineStr">
         <is>
           <t>业务方排期</t>
         </is>
       </c>
-    </row>
-    <row r="82" ht="22" customHeight="1" s="18">
-      <c r="A82" s="43" t="n"/>
-      <c r="B82" s="43" t="n"/>
-      <c r="C82" s="43" t="n"/>
-      <c r="D82" s="44" t="n"/>
-      <c r="E82" s="41" t="inlineStr">
-        <is>
-          <t>• 预演反馈裁决</t>
-        </is>
-      </c>
-      <c r="F82" s="43" t="n"/>
-      <c r="G82" s="43" t="n"/>
-    </row>
-    <row r="83" ht="22" customHeight="1" s="18">
-      <c r="A83" s="49" t="inlineStr">
-        <is>
-          <t>R2</t>
-        </is>
-      </c>
-      <c r="B83" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="C83" s="26" t="inlineStr">
-        <is>
-          <t>W11</t>
-        </is>
-      </c>
-      <c r="D83" s="45" t="inlineStr">
-        <is>
-          <t>DEV·Wade</t>
-        </is>
-      </c>
-      <c r="E83" s="41" t="inlineStr">
-        <is>
-          <t>• 全量回归（R1+R2）+ 安全终检（四门禁+渗透）</t>
-        </is>
-      </c>
-      <c r="F83" s="42" t="inlineStr">
-        <is>
-          <t>★ 全量对账 100%</t>
-        </is>
-      </c>
-      <c r="G83" s="29" t="inlineStr">
-        <is>
-          <t>渗透排期</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="22" customHeight="1" s="18">
-      <c r="A84" s="43" t="n"/>
-      <c r="B84" s="43" t="n"/>
-      <c r="C84" s="43" t="n"/>
-      <c r="D84" s="46" t="n"/>
-      <c r="E84" s="41" t="inlineStr">
-        <is>
-          <t>• 【01】全量迁移收尾 + 对账报告</t>
-        </is>
-      </c>
-      <c r="F84" s="43" t="n"/>
-      <c r="G84" s="43" t="n"/>
     </row>
     <row r="85" ht="22" customHeight="1" s="18">
       <c r="A85" s="43" t="n"/>
       <c r="B85" s="43" t="n"/>
       <c r="C85" s="43" t="n"/>
-      <c r="D85" s="46" t="n"/>
+      <c r="D85" s="44" t="n"/>
       <c r="E85" s="41" t="inlineStr">
         <is>
-          <t>• R2 发布包冻结 + 上线 Checklist v2</t>
+          <t>• 预演协调</t>
         </is>
       </c>
       <c r="F85" s="43" t="n"/>
@@ -4309,27 +4399,27 @@
       </c>
       <c r="B86" s="39" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="C86" s="26" t="inlineStr">
         <is>
-          <t>W11</t>
-        </is>
-      </c>
-      <c r="D86" s="47" t="inlineStr">
-        <is>
-          <t>QA</t>
+          <t>W12</t>
+        </is>
+      </c>
+      <c r="D86" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
         </is>
       </c>
       <c r="E86" s="41" t="inlineStr">
         <is>
-          <t>• 文档终审推进（7 套终稿）</t>
+          <t>• 全量回归（R1+R2）+ 功能收口</t>
         </is>
       </c>
       <c r="F86" s="42" t="inlineStr">
         <is>
-          <t>★ R2 就绪检查 100%</t>
+          <t>回归通过；R2 发布包 v1</t>
         </is>
       </c>
       <c r="G86" s="29" t="inlineStr"/>
@@ -4338,10 +4428,10 @@
       <c r="A87" s="43" t="n"/>
       <c r="B87" s="43" t="n"/>
       <c r="C87" s="43" t="n"/>
-      <c r="D87" s="48" t="n"/>
+      <c r="D87" s="46" t="n"/>
       <c r="E87" s="41" t="inlineStr">
         <is>
-          <t>• W11 末就绪检查组织（发布包/预演/文档/回退）</t>
+          <t>• 🤖 R2 发布包（增量/处置/加密/分层生产版）</t>
         </is>
       </c>
       <c r="F87" s="43" t="n"/>
@@ -4355,7 +4445,7 @@
       </c>
       <c r="B88" s="39" t="inlineStr">
         <is>
-          <t>Sprint 4</t>
+          <t>Sprint 5</t>
         </is>
       </c>
       <c r="C88" s="26" t="inlineStr">
@@ -4363,98 +4453,118 @@
           <t>W12</t>
         </is>
       </c>
-      <c r="D88" s="40" t="inlineStr">
-        <is>
-          <t>BA·Mandy</t>
+      <c r="D88" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
         </is>
       </c>
       <c r="E88" s="41" t="inlineStr">
         <is>
-          <t>• Go/No-Go #2 决策参与</t>
+          <t>• 文档冲刺：7 套进入终稿</t>
         </is>
       </c>
       <c r="F88" s="42" t="inlineStr">
         <is>
-          <t>★ UAT #2 签字</t>
-        </is>
-      </c>
-      <c r="G88" s="29" t="inlineStr">
-        <is>
-          <t>UAT 时间</t>
-        </is>
-      </c>
+          <t>文档 90%</t>
+        </is>
+      </c>
+      <c r="G88" s="29" t="inlineStr"/>
     </row>
     <row r="89" ht="22" customHeight="1" s="18">
       <c r="A89" s="43" t="n"/>
       <c r="B89" s="43" t="n"/>
       <c r="C89" s="43" t="n"/>
-      <c r="D89" s="44" t="n"/>
+      <c r="D89" s="48" t="n"/>
       <c r="E89" s="41" t="inlineStr">
         <is>
-          <t>• UAT #2 正式主持（签字）</t>
+          <t>• 🤖 审批材料起稿</t>
         </is>
       </c>
       <c r="F89" s="43" t="n"/>
       <c r="G89" s="43" t="n"/>
     </row>
     <row r="90" ht="22" customHeight="1" s="18">
-      <c r="A90" s="43" t="n"/>
-      <c r="B90" s="43" t="n"/>
-      <c r="C90" s="43" t="n"/>
-      <c r="D90" s="44" t="n"/>
+      <c r="A90" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B90" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C90" s="26" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="D90" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
+        </is>
+      </c>
       <c r="E90" s="41" t="inlineStr">
         <is>
-          <t>• 上线后反馈分诊</t>
-        </is>
-      </c>
-      <c r="F90" s="43" t="n"/>
-      <c r="G90" s="43" t="n"/>
+          <t>• UAT #2 预演主持（处置/Hold/脱敏/报表）</t>
+        </is>
+      </c>
+      <c r="F90" s="42" t="inlineStr">
+        <is>
+          <t>预演完成</t>
+        </is>
+      </c>
+      <c r="G90" s="29" t="inlineStr"/>
     </row>
     <row r="91" ht="22" customHeight="1" s="18">
-      <c r="A91" s="49" t="inlineStr">
+      <c r="A91" s="43" t="n"/>
+      <c r="B91" s="43" t="n"/>
+      <c r="C91" s="43" t="n"/>
+      <c r="D91" s="44" t="n"/>
+      <c r="E91" s="41" t="inlineStr">
+        <is>
+          <t>• 预演反馈裁决</t>
+        </is>
+      </c>
+      <c r="F91" s="43" t="n"/>
+      <c r="G91" s="43" t="n"/>
+    </row>
+    <row r="92" ht="22" customHeight="1" s="18">
+      <c r="A92" s="49" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B91" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="C91" s="26" t="inlineStr">
-        <is>
-          <t>W12</t>
-        </is>
-      </c>
-      <c r="D91" s="45" t="inlineStr">
+      <c r="B92" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C92" s="26" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="D92" s="45" t="inlineStr">
         <is>
           <t>DEV·Wade</t>
         </is>
       </c>
-      <c r="E91" s="41" t="inlineStr">
-        <is>
-          <t>• R2 生产发布（增量发布不中断 R1）</t>
-        </is>
-      </c>
-      <c r="F91" s="42" t="inlineStr">
-        <is>
-          <t>★ Go-Live #2</t>
-        </is>
-      </c>
-      <c r="G91" s="29" t="inlineStr"/>
-    </row>
-    <row r="92" ht="22" customHeight="1" s="18">
-      <c r="A92" s="43" t="n"/>
-      <c r="B92" s="43" t="n"/>
-      <c r="C92" s="43" t="n"/>
-      <c r="D92" s="46" t="n"/>
       <c r="E92" s="41" t="inlineStr">
         <is>
-          <t>• CC 生产全量迁移收尾+终版对账</t>
-        </is>
-      </c>
-      <c r="F92" s="43" t="n"/>
-      <c r="G92" s="43" t="n"/>
+          <t>• 回退演练+发布包冻结</t>
+        </is>
+      </c>
+      <c r="F92" s="42" t="inlineStr">
+        <is>
+          <t>终检通过；包冻结</t>
+        </is>
+      </c>
+      <c r="G92" s="29" t="inlineStr">
+        <is>
+          <t>渗透排期</t>
+        </is>
+      </c>
     </row>
     <row r="93" ht="22" customHeight="1" s="18">
       <c r="A93" s="43" t="n"/>
@@ -4463,61 +4573,57 @@
       <c r="D93" s="46" t="n"/>
       <c r="E93" s="41" t="inlineStr">
         <is>
-          <t>• P1 当日清 + 48h 值守 + 交付物 tag</t>
+          <t>• 安全终检（四门禁+渗透配合）</t>
         </is>
       </c>
       <c r="F93" s="43" t="n"/>
       <c r="G93" s="43" t="n"/>
     </row>
     <row r="94" ht="22" customHeight="1" s="18">
-      <c r="A94" s="49" t="inlineStr">
+      <c r="A94" s="43" t="n"/>
+      <c r="B94" s="43" t="n"/>
+      <c r="C94" s="43" t="n"/>
+      <c r="D94" s="46" t="n"/>
+      <c r="E94" s="41" t="inlineStr">
+        <is>
+          <t>• 迁移预跑+窗口预约</t>
+        </is>
+      </c>
+      <c r="F94" s="43" t="n"/>
+      <c r="G94" s="43" t="n"/>
+    </row>
+    <row r="95" ht="22" customHeight="1" s="18">
+      <c r="A95" s="49" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B94" s="39" t="inlineStr">
-        <is>
-          <t>Sprint 4</t>
-        </is>
-      </c>
-      <c r="C94" s="26" t="inlineStr">
-        <is>
-          <t>W12</t>
-        </is>
-      </c>
-      <c r="D94" s="47" t="inlineStr">
+      <c r="B95" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C95" s="26" t="inlineStr">
+        <is>
+          <t>W13</t>
+        </is>
+      </c>
+      <c r="D95" s="47" t="inlineStr">
         <is>
           <t>QA</t>
         </is>
       </c>
-      <c r="E94" s="41" t="inlineStr">
-        <is>
-          <t>• 审批材料提交（完整版）</t>
-        </is>
-      </c>
-      <c r="F94" s="42" t="inlineStr">
-        <is>
-          <t>★ Release 2 交付完成</t>
-        </is>
-      </c>
-      <c r="G94" s="29" t="inlineStr">
-        <is>
-          <t>审批受理</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="22" customHeight="1" s="18">
-      <c r="A95" s="43" t="n"/>
-      <c r="B95" s="43" t="n"/>
-      <c r="C95" s="43" t="n"/>
-      <c r="D95" s="48" t="n"/>
       <c r="E95" s="41" t="inlineStr">
         <is>
-          <t>• 文档终版归档（7 套）</t>
-        </is>
-      </c>
-      <c r="F95" s="43" t="n"/>
-      <c r="G95" s="43" t="n"/>
+          <t>• W13 末就绪检查组织（发布包/预演/文档/回退）</t>
+        </is>
+      </c>
+      <c r="F95" s="42" t="inlineStr">
+        <is>
+          <t>★ R2 就绪检查 100%</t>
+        </is>
+      </c>
+      <c r="G95" s="29" t="inlineStr"/>
     </row>
     <row r="96" ht="22" customHeight="1" s="18">
       <c r="A96" s="43" t="n"/>
@@ -4526,11 +4632,196 @@
       <c r="D96" s="48" t="n"/>
       <c r="E96" s="41" t="inlineStr">
         <is>
-          <t>• 上线验证与稳定性报告 → 项目结束</t>
+          <t>• 上线 Checklist v2</t>
         </is>
       </c>
       <c r="F96" s="43" t="n"/>
       <c r="G96" s="43" t="n"/>
+    </row>
+    <row r="97" ht="22" customHeight="1" s="18">
+      <c r="A97" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B97" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C97" s="26" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="D97" s="40" t="inlineStr">
+        <is>
+          <t>BA·Mandy</t>
+        </is>
+      </c>
+      <c r="E97" s="41" t="inlineStr">
+        <is>
+          <t>• Go/No-Go #2 决策参与</t>
+        </is>
+      </c>
+      <c r="F97" s="42" t="inlineStr">
+        <is>
+          <t>★ UAT #2 签字</t>
+        </is>
+      </c>
+      <c r="G97" s="29" t="inlineStr">
+        <is>
+          <t>UAT 时间</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1" s="18">
+      <c r="A98" s="43" t="n"/>
+      <c r="B98" s="43" t="n"/>
+      <c r="C98" s="43" t="n"/>
+      <c r="D98" s="44" t="n"/>
+      <c r="E98" s="41" t="inlineStr">
+        <is>
+          <t>• UAT #2 正式主持（签字）</t>
+        </is>
+      </c>
+      <c r="F98" s="43" t="n"/>
+      <c r="G98" s="43" t="n"/>
+    </row>
+    <row r="99" ht="22" customHeight="1" s="18">
+      <c r="A99" s="43" t="n"/>
+      <c r="B99" s="43" t="n"/>
+      <c r="C99" s="43" t="n"/>
+      <c r="D99" s="44" t="n"/>
+      <c r="E99" s="41" t="inlineStr">
+        <is>
+          <t>• 上线后反馈分诊</t>
+        </is>
+      </c>
+      <c r="F99" s="43" t="n"/>
+      <c r="G99" s="43" t="n"/>
+    </row>
+    <row r="100" ht="22" customHeight="1" s="18">
+      <c r="A100" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B100" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C100" s="26" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="D100" s="45" t="inlineStr">
+        <is>
+          <t>DEV·Wade</t>
+        </is>
+      </c>
+      <c r="E100" s="41" t="inlineStr">
+        <is>
+          <t>• R2 生产发布（增量不中断 R1）</t>
+        </is>
+      </c>
+      <c r="F100" s="42" t="inlineStr">
+        <is>
+          <t>★ Go-Live #2</t>
+        </is>
+      </c>
+      <c r="G100" s="29" t="inlineStr"/>
+    </row>
+    <row r="101" ht="22" customHeight="1" s="18">
+      <c r="A101" s="43" t="n"/>
+      <c r="B101" s="43" t="n"/>
+      <c r="C101" s="43" t="n"/>
+      <c r="D101" s="46" t="n"/>
+      <c r="E101" s="41" t="inlineStr">
+        <is>
+          <t>• CC 生产全量迁移收尾+终版对账</t>
+        </is>
+      </c>
+      <c r="F101" s="43" t="n"/>
+      <c r="G101" s="43" t="n"/>
+    </row>
+    <row r="102" ht="22" customHeight="1" s="18">
+      <c r="A102" s="43" t="n"/>
+      <c r="B102" s="43" t="n"/>
+      <c r="C102" s="43" t="n"/>
+      <c r="D102" s="46" t="n"/>
+      <c r="E102" s="41" t="inlineStr">
+        <is>
+          <t>• P1 当日清+48h 值守+交付物 tag</t>
+        </is>
+      </c>
+      <c r="F102" s="43" t="n"/>
+      <c r="G102" s="43" t="n"/>
+    </row>
+    <row r="103" ht="22" customHeight="1" s="18">
+      <c r="A103" s="49" t="inlineStr">
+        <is>
+          <t>R2</t>
+        </is>
+      </c>
+      <c r="B103" s="39" t="inlineStr">
+        <is>
+          <t>Sprint 5</t>
+        </is>
+      </c>
+      <c r="C103" s="26" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="D103" s="47" t="inlineStr">
+        <is>
+          <t>QA</t>
+        </is>
+      </c>
+      <c r="E103" s="41" t="inlineStr">
+        <is>
+          <t>• 审批材料提交（完整版）</t>
+        </is>
+      </c>
+      <c r="F103" s="42" t="inlineStr">
+        <is>
+          <t>★ Release 2 交付完成</t>
+        </is>
+      </c>
+      <c r="G103" s="29" t="inlineStr">
+        <is>
+          <t>审批受理</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1" s="18">
+      <c r="A104" s="43" t="n"/>
+      <c r="B104" s="43" t="n"/>
+      <c r="C104" s="43" t="n"/>
+      <c r="D104" s="48" t="n"/>
+      <c r="E104" s="41" t="inlineStr">
+        <is>
+          <t>• 文档终版归档（7 套）</t>
+        </is>
+      </c>
+      <c r="F104" s="43" t="n"/>
+      <c r="G104" s="43" t="n"/>
+    </row>
+    <row r="105" ht="22" customHeight="1" s="18">
+      <c r="A105" s="43" t="n"/>
+      <c r="B105" s="43" t="n"/>
+      <c r="C105" s="43" t="n"/>
+      <c r="D105" s="48" t="n"/>
+      <c r="E105" s="41" t="inlineStr">
+        <is>
+          <t>• 稳定性报告 → 项目结束</t>
+        </is>
+      </c>
+      <c r="F105" s="43" t="n"/>
+      <c r="G105" s="43" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>